<commit_message>
update Rally1 and HSC damping
</commit_message>
<xml_diff>
--- a/docs/damping_curve_RAx5.xlsx
+++ b/docs/damping_curve_RAx5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D45ABE-D6F8-4F9D-BC3B-4F991366B8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8BB36E-8F5B-4273-83D4-C74ED369B666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalog" sheetId="8" r:id="rId1"/>
@@ -1797,11 +1797,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1816,7 +1816,7 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1834,10 +1834,10 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1855,10 +1855,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1993,40 +1993,61 @@
     <xf numFmtId="0" fontId="78" fillId="69" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="44" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="45" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="24" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="25" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="24" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="30" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="31" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="41" fillId="32" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="33" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="41" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2038,38 +2059,14 @@
     <xf numFmtId="0" fontId="52" fillId="43" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="30" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="53" fillId="44" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="31" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="54" fillId="45" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="25" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="46" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3359,31 +3356,31 @@
                   <c:v>1268.4000000000001</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1398.3999999999999</c:v>
+                  <c:v>1390.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1552.4</c:v>
+                  <c:v>1524.4</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1706.3999999999999</c:v>
+                  <c:v>1658.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1860.4</c:v>
+                  <c:v>1792.4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2014.4</c:v>
+                  <c:v>1926.4</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2168.3999999999996</c:v>
+                  <c:v>2060.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2322.4</c:v>
+                  <c:v>2194.4</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2476.3999999999996</c:v>
+                  <c:v>2328.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2630.4</c:v>
+                  <c:v>2462.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3535,31 +3532,31 @@
                   <c:v>1268.4000000000001</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1396.3999999999999</c:v>
+                  <c:v>1394.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1580.4</c:v>
+                  <c:v>1568.4</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1764.3999999999999</c:v>
+                  <c:v>1742.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1948.4</c:v>
+                  <c:v>1916.4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2132.4</c:v>
+                  <c:v>2090.4</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2316.3999999999996</c:v>
+                  <c:v>2264.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2500.4</c:v>
+                  <c:v>2438.4</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2684.3999999999996</c:v>
+                  <c:v>2612.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2868.4</c:v>
+                  <c:v>2786.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3890,28 +3887,28 @@
                   <c:v>1382.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1600.4</c:v>
+                  <c:v>1608.4</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1844.3999999999999</c:v>
+                  <c:v>1862.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2088.4</c:v>
+                  <c:v>2116.4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2332.4</c:v>
+                  <c:v>2370.4</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2576.3999999999996</c:v>
+                  <c:v>2624.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2820.4</c:v>
+                  <c:v>2878.4</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3064.3999999999996</c:v>
+                  <c:v>3132.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3308.4</c:v>
+                  <c:v>3386.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4066,28 +4063,28 @@
                   <c:v>1382.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1592.4</c:v>
+                  <c:v>1604.4</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1866.3999999999996</c:v>
+                  <c:v>1898.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2140.4</c:v>
+                  <c:v>2192.4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2414.4</c:v>
+                  <c:v>2486.4000000000005</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2688.3999999999996</c:v>
+                  <c:v>2780.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2962.4</c:v>
+                  <c:v>3074.4</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3236.3999999999996</c:v>
+                  <c:v>3368.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3510.4</c:v>
+                  <c:v>3662.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5512,31 +5509,31 @@
                   <c:v>660.00000000000011</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>736</c:v>
+                  <c:v>728</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>836</c:v>
+                  <c:v>808</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>936</c:v>
+                  <c:v>888</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1036</c:v>
+                  <c:v>968</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1136.0000000000002</c:v>
+                  <c:v>1048.0000000000002</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1236</c:v>
+                  <c:v>1128</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1336</c:v>
+                  <c:v>1208</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1436</c:v>
+                  <c:v>1288</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1536</c:v>
+                  <c:v>1368</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5688,31 +5685,31 @@
                   <c:v>970.65000000000009</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1072.4000000000001</c:v>
+                  <c:v>1070.4000000000001</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1230.1500000000001</c:v>
+                  <c:v>1218.1500000000001</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1387.9</c:v>
+                  <c:v>1365.9</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1545.65</c:v>
+                  <c:v>1513.65</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1703.4</c:v>
+                  <c:v>1661.4</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1861.1499999999999</c:v>
+                  <c:v>1809.1499999999999</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2018.9</c:v>
+                  <c:v>1956.9</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2176.6499999999996</c:v>
+                  <c:v>2104.6499999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2334.4</c:v>
+                  <c:v>2252.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6043,28 +6040,28 @@
                   <c:v>1692</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1934.75</c:v>
+                  <c:v>1942.75</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2203.5</c:v>
+                  <c:v>2221.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2472.25</c:v>
+                  <c:v>2500.25</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2741</c:v>
+                  <c:v>2779</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3009.75</c:v>
+                  <c:v>3057.75</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3278.5</c:v>
+                  <c:v>3336.5</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3547.25</c:v>
+                  <c:v>3615.25</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3816</c:v>
+                  <c:v>3894</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6219,28 +6216,28 @@
                   <c:v>1987.2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2245.1999999999998</c:v>
+                  <c:v>2257.1999999999998</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2567.1999999999998</c:v>
+                  <c:v>2599.1999999999998</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2889.2</c:v>
+                  <c:v>2941.2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3211.2000000000003</c:v>
+                  <c:v>3283.2000000000007</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3533.2</c:v>
+                  <c:v>3625.2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3855.2000000000003</c:v>
+                  <c:v>3967.2000000000003</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4177.2</c:v>
+                  <c:v>4309.2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>4499.2</c:v>
+                  <c:v>4651.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7664,14 +7661,14 @@
     </row>
     <row r="2" spans="1:8" ht="35" customHeight="1">
       <c r="A2" s="6"/>
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:8" ht="25" customHeight="1">
@@ -7722,7 +7719,7 @@
     </row>
     <row r="6" spans="1:8" ht="31" customHeight="1">
       <c r="A6" s="6"/>
-      <c r="B6" s="83" t="s">
+      <c r="B6" s="70" t="s">
         <v>77</v>
       </c>
       <c r="C6" s="6"/>
@@ -7742,7 +7739,7 @@
     </row>
     <row r="7" spans="1:8" ht="31" customHeight="1">
       <c r="A7" s="6"/>
-      <c r="B7" s="83"/>
+      <c r="B7" s="70"/>
       <c r="C7" s="6"/>
       <c r="D7" s="12" t="s">
         <v>79</v>
@@ -7876,30 +7873,30 @@
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="80"/>
-      <c r="G15" s="80"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" ht="22" customHeight="1">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
-      <c r="D16" s="80"/>
-      <c r="E16" s="80"/>
-      <c r="F16" s="80"/>
-      <c r="G16" s="80"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="67"/>
       <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:8" ht="22" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
-      <c r="G17" s="80"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="67"/>
+      <c r="G17" s="67"/>
       <c r="H17" s="6"/>
     </row>
     <row r="18" spans="1:8" ht="25" customHeight="1">
@@ -7990,20 +7987,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="22"/>
       <c r="O2" s="1"/>
     </row>
@@ -8033,15 +8030,15 @@
         <v>95</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8072,7 +8069,7 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="73" t="s">
+      <c r="F6" s="71" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="72"/>
@@ -8116,16 +8113,16 @@
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="68" t="s">
+      <c r="F8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="76"/>
-      <c r="H8" s="76"/>
-      <c r="I8" s="88">
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="74">
         <f>IF(C18="OK",Samples!F165*MIN(C10,Samples!G165)+Samples!I165*MAX(0,C10-Samples!G165)+Samples!J165*MAX(0,C10-Samples!K165),"检查输入")</f>
-        <v>3181.44</v>
-      </c>
-      <c r="J8" s="89"/>
+        <v>3213.12</v>
+      </c>
+      <c r="J8" s="75"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -8163,16 +8160,16 @@
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="68" t="s">
+      <c r="F10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="88">
+      <c r="G10" s="73"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="74">
         <f>IF(C18="OK",Samples!M165*MIN(C10,Samples!N165)+Samples!P165*MAX(0,C10-Samples!N165),"检查输入")</f>
         <v>1832</v>
       </c>
-      <c r="J10" s="89"/>
+      <c r="J10" s="75"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -8224,7 +8221,7 @@
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="73" t="s">
+      <c r="F13" s="71" t="s">
         <v>47</v>
       </c>
       <c r="G13" s="72"/>
@@ -8248,11 +8245,11 @@
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="86" t="s">
+      <c r="F14" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="75"/>
-      <c r="H14" s="75"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
       <c r="I14" s="32">
         <f>Samples!F165</f>
         <v>2400</v>
@@ -8277,11 +8274,11 @@
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="76" t="s">
+      <c r="F15" s="73" t="s">
         <v>26</v>
       </c>
-      <c r="G15" s="69"/>
-      <c r="H15" s="69"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
       <c r="I15" s="33">
         <f>Samples!I165</f>
         <v>2280</v>
@@ -8301,14 +8298,14 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="74" t="s">
+      <c r="F16" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="75"/>
-      <c r="H16" s="75"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
       <c r="I16" s="32">
         <f>Samples!J165</f>
-        <v>2240</v>
+        <v>2320</v>
       </c>
       <c r="J16" s="23" t="s">
         <v>11</v>
@@ -8325,14 +8322,14 @@
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="68" t="s">
+      <c r="F17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="69"/>
-      <c r="H17" s="69"/>
+      <c r="G17" s="78"/>
+      <c r="H17" s="78"/>
       <c r="I17" s="33">
         <f>Samples!L165</f>
-        <v>4520</v>
+        <v>4600</v>
       </c>
       <c r="J17" s="26" t="s">
         <v>11</v>
@@ -8371,11 +8368,11 @@
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="86" t="s">
+      <c r="F19" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="G19" s="75"/>
-      <c r="H19" s="75"/>
+      <c r="G19" s="77"/>
+      <c r="H19" s="77"/>
       <c r="I19" s="32">
         <f>Samples!M165</f>
         <v>2000</v>
@@ -8395,11 +8392,11 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="76" t="s">
+      <c r="F20" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="69"/>
-      <c r="H20" s="69"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="78"/>
       <c r="I20" s="33">
         <f>Samples!P165</f>
         <v>1760</v>
@@ -8436,11 +8433,11 @@
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="74" t="s">
+      <c r="F22" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="G22" s="75"/>
-      <c r="H22" s="75"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
       <c r="I22" s="35">
         <f>Samples!G165</f>
         <v>0.12</v>
@@ -8460,11 +8457,11 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="68" t="s">
+      <c r="F23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="69"/>
-      <c r="H23" s="69"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
       <c r="I23" s="36">
         <f>Samples!K165</f>
         <v>0.60399999999999998</v>
@@ -8484,11 +8481,11 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="86" t="s">
+      <c r="F24" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="G24" s="75"/>
-      <c r="H24" s="75"/>
+      <c r="G24" s="77"/>
+      <c r="H24" s="77"/>
       <c r="I24" s="35">
         <f>Samples!N165</f>
         <v>0.3</v>
@@ -8538,20 +8535,20 @@
     </row>
     <row r="27" spans="1:15" ht="23.15" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="84" t="s">
+      <c r="B27" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="C27" s="85"/>
-      <c r="D27" s="85"/>
-      <c r="E27" s="85"/>
-      <c r="F27" s="85"/>
-      <c r="G27" s="85"/>
-      <c r="H27" s="85"/>
-      <c r="I27" s="85"/>
-      <c r="J27" s="85"/>
-      <c r="K27" s="85"/>
-      <c r="L27" s="85"/>
-      <c r="M27" s="85"/>
+      <c r="C27" s="81"/>
+      <c r="D27" s="81"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="81"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
+      <c r="I27" s="81"/>
+      <c r="J27" s="81"/>
+      <c r="K27" s="81"/>
+      <c r="L27" s="81"/>
+      <c r="M27" s="81"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
     </row>
@@ -8812,6 +8809,17 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B27:M27"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E4:M4"/>
     <mergeCell ref="F6:J6"/>
@@ -8819,17 +8827,6 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I10:J10"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="B27:M27"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <dataValidations count="5">
@@ -8886,20 +8883,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="22"/>
       <c r="O2" s="1"/>
     </row>
@@ -8929,15 +8926,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8967,15 +8964,15 @@
         <v>-10</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9559,18 +9556,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="90"/>
-      <c r="C41" s="90"/>
-      <c r="D41" s="90"/>
-      <c r="E41" s="90"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="90"/>
-      <c r="H41" s="90"/>
-      <c r="I41" s="90"/>
-      <c r="J41" s="90"/>
-      <c r="K41" s="90"/>
-      <c r="L41" s="90"/>
-      <c r="M41" s="90"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="66"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
+      <c r="H41" s="66"/>
+      <c r="I41" s="66"/>
+      <c r="J41" s="66"/>
+      <c r="K41" s="66"/>
+      <c r="L41" s="66"/>
+      <c r="M41" s="66"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -9644,20 +9641,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="22"/>
       <c r="O2" s="1"/>
     </row>
@@ -9687,15 +9684,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -9725,15 +9722,15 @@
         <v>-12</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -10317,18 +10314,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="90"/>
-      <c r="C41" s="90"/>
-      <c r="D41" s="90"/>
-      <c r="E41" s="90"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="90"/>
-      <c r="H41" s="90"/>
-      <c r="I41" s="90"/>
-      <c r="J41" s="90"/>
-      <c r="K41" s="90"/>
-      <c r="L41" s="90"/>
-      <c r="M41" s="90"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="66"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
+      <c r="H41" s="66"/>
+      <c r="I41" s="66"/>
+      <c r="J41" s="66"/>
+      <c r="K41" s="66"/>
+      <c r="L41" s="66"/>
+      <c r="M41" s="66"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -10402,20 +10399,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="22"/>
       <c r="O2" s="1"/>
     </row>
@@ -10445,15 +10442,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -10476,18 +10473,18 @@
     </row>
     <row r="6" spans="1:15" ht="28" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -11071,18 +11068,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="90"/>
-      <c r="C41" s="90"/>
-      <c r="D41" s="90"/>
-      <c r="E41" s="90"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="90"/>
-      <c r="H41" s="90"/>
-      <c r="I41" s="90"/>
-      <c r="J41" s="90"/>
-      <c r="K41" s="90"/>
-      <c r="L41" s="90"/>
-      <c r="M41" s="90"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="66"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
+      <c r="H41" s="66"/>
+      <c r="I41" s="66"/>
+      <c r="J41" s="66"/>
+      <c r="K41" s="66"/>
+      <c r="L41" s="66"/>
+      <c r="M41" s="66"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -11152,20 +11149,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="22"/>
       <c r="O2" s="1"/>
     </row>
@@ -11195,15 +11192,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -11226,18 +11223,18 @@
     </row>
     <row r="6" spans="1:15" ht="28" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -11821,18 +11818,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="90"/>
-      <c r="C41" s="90"/>
-      <c r="D41" s="90"/>
-      <c r="E41" s="90"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="90"/>
-      <c r="H41" s="90"/>
-      <c r="I41" s="90"/>
-      <c r="J41" s="90"/>
-      <c r="K41" s="90"/>
-      <c r="L41" s="90"/>
-      <c r="M41" s="90"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="66"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
+      <c r="H41" s="66"/>
+      <c r="I41" s="66"/>
+      <c r="J41" s="66"/>
+      <c r="K41" s="66"/>
+      <c r="L41" s="66"/>
+      <c r="M41" s="66"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -11906,40 +11903,40 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="24" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="82" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
+      <c r="K3" s="83"/>
+      <c r="L3" s="83"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="83"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" ht="28" customHeight="1">
@@ -12289,21 +12286,21 @@
         <v>11</v>
       </c>
       <c r="D13" s="27">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="E13" s="41">
         <f>(D13+F13)/2</f>
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="F13" s="27">
         <v>2000</v>
       </c>
       <c r="G13" s="41">
         <f>(F13+H13)/2</f>
-        <v>2600</v>
+        <v>2800</v>
       </c>
       <c r="H13" s="27">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="27">
@@ -12609,7 +12606,7 @@
     </row>
     <row r="22" spans="1:15" ht="32" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="73" t="s">
+      <c r="B22" s="71" t="s">
         <v>52</v>
       </c>
       <c r="C22" s="72"/>
@@ -12628,54 +12625,54 @@
     </row>
     <row r="23" spans="1:15" ht="29" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="74" t="s">
+      <c r="B23" s="79" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="75"/>
+      <c r="C23" s="77"/>
       <c r="D23" s="29">
         <v>24</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="77" t="s">
+      <c r="F23" s="84" t="s">
         <v>85</v>
       </c>
-      <c r="G23" s="78"/>
-      <c r="H23" s="78"/>
-      <c r="I23" s="78"/>
-      <c r="J23" s="78"/>
-      <c r="K23" s="78"/>
-      <c r="L23" s="78"/>
-      <c r="M23" s="78"/>
-      <c r="N23" s="78"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="85"/>
+      <c r="J23" s="85"/>
+      <c r="K23" s="85"/>
+      <c r="L23" s="85"/>
+      <c r="M23" s="85"/>
+      <c r="N23" s="85"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="29" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="68" t="s">
+      <c r="B24" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C24" s="69"/>
+      <c r="C24" s="78"/>
       <c r="D24" s="31">
         <v>20</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="78"/>
-      <c r="G24" s="78"/>
-      <c r="H24" s="78"/>
-      <c r="I24" s="78"/>
-      <c r="J24" s="78"/>
-      <c r="K24" s="78"/>
-      <c r="L24" s="78"/>
-      <c r="M24" s="78"/>
-      <c r="N24" s="78"/>
+      <c r="F24" s="85"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="85"/>
+      <c r="J24" s="85"/>
+      <c r="K24" s="85"/>
+      <c r="L24" s="85"/>
+      <c r="M24" s="85"/>
+      <c r="N24" s="85"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="29" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="74" t="s">
+      <c r="B25" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="75"/>
+      <c r="C25" s="77"/>
       <c r="D25" s="29">
         <v>40</v>
       </c>
@@ -12693,33 +12690,33 @@
     </row>
     <row r="26" spans="1:15" ht="29" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="76" t="s">
+      <c r="B26" s="73" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="69"/>
+      <c r="C26" s="78"/>
       <c r="D26" s="31">
         <v>60</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="79" t="s">
+      <c r="F26" s="86" t="s">
         <v>87</v>
       </c>
-      <c r="G26" s="71"/>
-      <c r="H26" s="71"/>
-      <c r="I26" s="71"/>
-      <c r="J26" s="71"/>
-      <c r="K26" s="71"/>
-      <c r="L26" s="71"/>
-      <c r="M26" s="71"/>
-      <c r="N26" s="71"/>
+      <c r="G26" s="83"/>
+      <c r="H26" s="83"/>
+      <c r="I26" s="83"/>
+      <c r="J26" s="83"/>
+      <c r="K26" s="83"/>
+      <c r="L26" s="83"/>
+      <c r="M26" s="83"/>
+      <c r="N26" s="83"/>
       <c r="O26" s="1"/>
     </row>
     <row r="27" spans="1:15" ht="29" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="68" t="s">
+      <c r="B27" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C27" s="69"/>
+      <c r="C27" s="78"/>
       <c r="D27" s="31">
         <v>10</v>
       </c>
@@ -12737,21 +12734,21 @@
     </row>
     <row r="28" spans="1:15" ht="24" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="65" t="s">
+      <c r="B28" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="66"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
-      <c r="F28" s="66"/>
-      <c r="G28" s="66"/>
-      <c r="H28" s="66"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="66"/>
-      <c r="K28" s="66"/>
-      <c r="L28" s="66"/>
-      <c r="M28" s="66"/>
-      <c r="N28" s="66"/>
+      <c r="C28" s="88"/>
+      <c r="D28" s="88"/>
+      <c r="E28" s="88"/>
+      <c r="F28" s="88"/>
+      <c r="G28" s="88"/>
+      <c r="H28" s="88"/>
+      <c r="I28" s="88"/>
+      <c r="J28" s="88"/>
+      <c r="K28" s="88"/>
+      <c r="L28" s="88"/>
+      <c r="M28" s="88"/>
+      <c r="N28" s="88"/>
       <c r="O28" s="1"/>
     </row>
     <row r="29" spans="1:15" ht="23.15" customHeight="1">
@@ -12773,19 +12770,19 @@
     </row>
     <row r="30" spans="1:15" ht="31" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="67"/>
-      <c r="C30" s="67"/>
-      <c r="D30" s="67"/>
-      <c r="E30" s="67"/>
-      <c r="F30" s="67"/>
-      <c r="G30" s="67"/>
-      <c r="H30" s="67"/>
-      <c r="I30" s="67"/>
-      <c r="J30" s="67"/>
-      <c r="K30" s="67"/>
-      <c r="L30" s="67"/>
-      <c r="M30" s="67"/>
-      <c r="N30" s="67"/>
+      <c r="B30" s="89"/>
+      <c r="C30" s="89"/>
+      <c r="D30" s="89"/>
+      <c r="E30" s="89"/>
+      <c r="F30" s="89"/>
+      <c r="G30" s="89"/>
+      <c r="H30" s="89"/>
+      <c r="I30" s="89"/>
+      <c r="J30" s="89"/>
+      <c r="K30" s="89"/>
+      <c r="L30" s="89"/>
+      <c r="M30" s="89"/>
+      <c r="N30" s="89"/>
       <c r="O30" s="1"/>
     </row>
     <row r="31" spans="1:15" ht="23.15" customHeight="1">
@@ -12977,6 +12974,14 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B33:N33"/>
+    <mergeCell ref="B34:N34"/>
+    <mergeCell ref="B35:N35"/>
+    <mergeCell ref="B28:N28"/>
+    <mergeCell ref="B29:N29"/>
+    <mergeCell ref="B30:N30"/>
+    <mergeCell ref="B31:N31"/>
+    <mergeCell ref="B32:N32"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B3:N3"/>
@@ -12989,14 +12994,6 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="F23:N24"/>
     <mergeCell ref="F26:N26"/>
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="B34:N34"/>
-    <mergeCell ref="B35:N35"/>
-    <mergeCell ref="B28:N28"/>
-    <mergeCell ref="B29:N29"/>
-    <mergeCell ref="B30:N30"/>
-    <mergeCell ref="B31:N31"/>
-    <mergeCell ref="B32:N32"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13018,29 +13015,29 @@
   <sheetData>
     <row r="1" spans="1:22" ht="32" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="91" t="s">
+      <c r="B1" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="91"/>
-      <c r="L1" s="91"/>
-      <c r="M1" s="91"/>
-      <c r="N1" s="91"/>
-      <c r="O1" s="91"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="92"/>
-      <c r="T1" s="92"/>
-      <c r="U1" s="92"/>
-      <c r="V1" s="92"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
     </row>
     <row r="2" spans="1:22" ht="22" customHeight="1">
       <c r="A2" s="1"/>
@@ -14711,29 +14708,29 @@
     </row>
     <row r="41" spans="1:22" ht="32" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="91" t="s">
+      <c r="B41" s="90" t="s">
         <v>91</v>
       </c>
-      <c r="C41" s="91"/>
-      <c r="D41" s="91"/>
-      <c r="E41" s="91"/>
-      <c r="F41" s="91"/>
-      <c r="G41" s="91"/>
-      <c r="H41" s="91"/>
-      <c r="I41" s="91"/>
-      <c r="J41" s="91"/>
-      <c r="K41" s="91"/>
-      <c r="L41" s="91"/>
-      <c r="M41" s="91"/>
-      <c r="N41" s="91"/>
-      <c r="O41" s="91"/>
-      <c r="P41" s="92"/>
-      <c r="Q41" s="92"/>
-      <c r="R41" s="92"/>
-      <c r="S41" s="92"/>
-      <c r="T41" s="92"/>
-      <c r="U41" s="92"/>
-      <c r="V41" s="92"/>
+      <c r="C41" s="90"/>
+      <c r="D41" s="90"/>
+      <c r="E41" s="90"/>
+      <c r="F41" s="90"/>
+      <c r="G41" s="90"/>
+      <c r="H41" s="90"/>
+      <c r="I41" s="90"/>
+      <c r="J41" s="90"/>
+      <c r="K41" s="90"/>
+      <c r="L41" s="90"/>
+      <c r="M41" s="90"/>
+      <c r="N41" s="90"/>
+      <c r="O41" s="90"/>
+      <c r="P41" s="91"/>
+      <c r="Q41" s="91"/>
+      <c r="R41" s="91"/>
+      <c r="S41" s="91"/>
+      <c r="T41" s="91"/>
+      <c r="U41" s="91"/>
+      <c r="V41" s="91"/>
     </row>
     <row r="42" spans="1:22" ht="22" customHeight="1">
       <c r="A42" s="1"/>
@@ -14882,7 +14879,7 @@
       </c>
       <c r="J45" s="50">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R45)+(INDEX(Parameters!$J$13:$N$13,1,R45+1)-INDEX(Parameters!$J$13:$N$13,1,R45))*U45,INDEX(Parameters!$D$13:$H$13,1,R45)+(INDEX(Parameters!$D$13:$H$13,1,R45+1)-INDEX(Parameters!$D$13:$H$13,1,R45))*U45)</f>
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="K45" s="50">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R45)+(INDEX(Parameters!$D$14:$H$14,1,R45+1)-INDEX(Parameters!$D$14:$H$14,1,R45))*U45)</f>
@@ -14890,7 +14887,7 @@
       </c>
       <c r="L45" s="50">
         <f>I45+J45</f>
-        <v>3080</v>
+        <v>2680</v>
       </c>
       <c r="M45" s="50">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S45)+(INDEX(Parameters!$J$17:$N$17,1,S45+1)-INDEX(Parameters!$J$17:$N$17,1,S45))*V45,INDEX(Parameters!$D$17:$H$17,1,S45)+(INDEX(Parameters!$D$17:$H$17,1,S45+1)-INDEX(Parameters!$D$17:$H$17,1,S45))*V45)</f>
@@ -14968,7 +14965,7 @@
       </c>
       <c r="J46" s="52">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R46)+(INDEX(Parameters!$J$13:$N$13,1,R46+1)-INDEX(Parameters!$J$13:$N$13,1,R46))*U46,INDEX(Parameters!$D$13:$H$13,1,R46)+(INDEX(Parameters!$D$13:$H$13,1,R46+1)-INDEX(Parameters!$D$13:$H$13,1,R46))*U46)</f>
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="K46" s="52">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R46)+(INDEX(Parameters!$D$14:$H$14,1,R46+1)-INDEX(Parameters!$D$14:$H$14,1,R46))*U46)</f>
@@ -14976,7 +14973,7 @@
       </c>
       <c r="L46" s="52">
         <f>I46+J46</f>
-        <v>3680</v>
+        <v>3480</v>
       </c>
       <c r="M46" s="52">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S46)+(INDEX(Parameters!$J$17:$N$17,1,S46+1)-INDEX(Parameters!$J$17:$N$17,1,S46))*V46,INDEX(Parameters!$D$17:$H$17,1,S46)+(INDEX(Parameters!$D$17:$H$17,1,S46+1)-INDEX(Parameters!$D$17:$H$17,1,S46))*V46)</f>
@@ -15140,7 +15137,7 @@
       </c>
       <c r="J48" s="52">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R48)+(INDEX(Parameters!$J$13:$N$13,1,R48+1)-INDEX(Parameters!$J$13:$N$13,1,R48))*U48,INDEX(Parameters!$D$13:$H$13,1,R48)+(INDEX(Parameters!$D$13:$H$13,1,R48+1)-INDEX(Parameters!$D$13:$H$13,1,R48))*U48)</f>
-        <v>2600</v>
+        <v>2800</v>
       </c>
       <c r="K48" s="52">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R48)+(INDEX(Parameters!$D$14:$H$14,1,R48+1)-INDEX(Parameters!$D$14:$H$14,1,R48))*U48)</f>
@@ -15148,7 +15145,7 @@
       </c>
       <c r="L48" s="52">
         <f>I48+J48</f>
-        <v>4880</v>
+        <v>5080</v>
       </c>
       <c r="M48" s="52">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S48)+(INDEX(Parameters!$J$17:$N$17,1,S48+1)-INDEX(Parameters!$J$17:$N$17,1,S48))*V48,INDEX(Parameters!$D$17:$H$17,1,S48)+(INDEX(Parameters!$D$17:$H$17,1,S48+1)-INDEX(Parameters!$D$17:$H$17,1,S48))*V48)</f>
@@ -15226,7 +15223,7 @@
       </c>
       <c r="J49" s="50">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R49)+(INDEX(Parameters!$J$13:$N$13,1,R49+1)-INDEX(Parameters!$J$13:$N$13,1,R49))*U49,INDEX(Parameters!$D$13:$H$13,1,R49)+(INDEX(Parameters!$D$13:$H$13,1,R49+1)-INDEX(Parameters!$D$13:$H$13,1,R49))*U49)</f>
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="K49" s="50">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R49)+(INDEX(Parameters!$D$14:$H$14,1,R49+1)-INDEX(Parameters!$D$14:$H$14,1,R49))*U49)</f>
@@ -15234,7 +15231,7 @@
       </c>
       <c r="L49" s="50">
         <f>I49+J49</f>
-        <v>5480</v>
+        <v>5880</v>
       </c>
       <c r="M49" s="50">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S49)+(INDEX(Parameters!$J$17:$N$17,1,S49+1)-INDEX(Parameters!$J$17:$N$17,1,S49))*V49,INDEX(Parameters!$D$17:$H$17,1,S49)+(INDEX(Parameters!$D$17:$H$17,1,S49+1)-INDEX(Parameters!$D$17:$H$17,1,S49))*V49)</f>
@@ -15872,11 +15869,11 @@
       </c>
       <c r="C66" s="59">
         <f t="shared" si="5"/>
-        <v>1398.3999999999999</v>
+        <v>1390.3999999999999</v>
       </c>
       <c r="D66" s="59">
         <f t="shared" si="6"/>
-        <v>1396.3999999999999</v>
+        <v>1394.3999999999999</v>
       </c>
       <c r="E66" s="59">
         <f t="shared" si="7"/>
@@ -15912,11 +15909,11 @@
       </c>
       <c r="C67" s="60">
         <f t="shared" si="5"/>
-        <v>1552.4</v>
+        <v>1524.4</v>
       </c>
       <c r="D67" s="60">
         <f t="shared" si="6"/>
-        <v>1580.4</v>
+        <v>1568.4</v>
       </c>
       <c r="E67" s="60">
         <f t="shared" si="7"/>
@@ -15924,11 +15921,11 @@
       </c>
       <c r="F67" s="60">
         <f t="shared" si="8"/>
-        <v>1600.4</v>
+        <v>1608.4</v>
       </c>
       <c r="G67" s="60">
         <f t="shared" si="9"/>
-        <v>1592.4</v>
+        <v>1604.4</v>
       </c>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
@@ -15952,11 +15949,11 @@
       </c>
       <c r="C68" s="59">
         <f t="shared" si="5"/>
-        <v>1706.3999999999999</v>
+        <v>1658.3999999999999</v>
       </c>
       <c r="D68" s="59">
         <f t="shared" si="6"/>
-        <v>1764.3999999999999</v>
+        <v>1742.3999999999999</v>
       </c>
       <c r="E68" s="59">
         <f t="shared" si="7"/>
@@ -15964,11 +15961,11 @@
       </c>
       <c r="F68" s="59">
         <f t="shared" si="8"/>
-        <v>1844.3999999999999</v>
+        <v>1862.3999999999999</v>
       </c>
       <c r="G68" s="59">
         <f t="shared" si="9"/>
-        <v>1866.3999999999996</v>
+        <v>1898.3999999999996</v>
       </c>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
@@ -15992,11 +15989,11 @@
       </c>
       <c r="C69" s="60">
         <f t="shared" si="5"/>
-        <v>1860.4</v>
+        <v>1792.4</v>
       </c>
       <c r="D69" s="60">
         <f t="shared" si="6"/>
-        <v>1948.4</v>
+        <v>1916.4</v>
       </c>
       <c r="E69" s="60">
         <f t="shared" si="7"/>
@@ -16004,11 +16001,11 @@
       </c>
       <c r="F69" s="60">
         <f t="shared" si="8"/>
-        <v>2088.4</v>
+        <v>2116.4</v>
       </c>
       <c r="G69" s="60">
         <f t="shared" si="9"/>
-        <v>2140.4</v>
+        <v>2192.4</v>
       </c>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
@@ -16032,11 +16029,11 @@
       </c>
       <c r="C70" s="59">
         <f t="shared" si="5"/>
-        <v>2014.4</v>
+        <v>1926.4</v>
       </c>
       <c r="D70" s="59">
         <f t="shared" si="6"/>
-        <v>2132.4</v>
+        <v>2090.4</v>
       </c>
       <c r="E70" s="59">
         <f t="shared" si="7"/>
@@ -16044,11 +16041,11 @@
       </c>
       <c r="F70" s="59">
         <f t="shared" si="8"/>
-        <v>2332.4</v>
+        <v>2370.4</v>
       </c>
       <c r="G70" s="59">
         <f t="shared" si="9"/>
-        <v>2414.4</v>
+        <v>2486.4000000000005</v>
       </c>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
@@ -16072,11 +16069,11 @@
       </c>
       <c r="C71" s="60">
         <f t="shared" si="5"/>
-        <v>2168.3999999999996</v>
+        <v>2060.3999999999996</v>
       </c>
       <c r="D71" s="60">
         <f t="shared" si="6"/>
-        <v>2316.3999999999996</v>
+        <v>2264.3999999999996</v>
       </c>
       <c r="E71" s="60">
         <f t="shared" si="7"/>
@@ -16084,11 +16081,11 @@
       </c>
       <c r="F71" s="60">
         <f t="shared" si="8"/>
-        <v>2576.3999999999996</v>
+        <v>2624.3999999999996</v>
       </c>
       <c r="G71" s="60">
         <f t="shared" si="9"/>
-        <v>2688.3999999999996</v>
+        <v>2780.3999999999996</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
@@ -16112,11 +16109,11 @@
       </c>
       <c r="C72" s="59">
         <f t="shared" si="5"/>
-        <v>2322.4</v>
+        <v>2194.4</v>
       </c>
       <c r="D72" s="59">
         <f t="shared" si="6"/>
-        <v>2500.4</v>
+        <v>2438.4</v>
       </c>
       <c r="E72" s="59">
         <f t="shared" si="7"/>
@@ -16124,11 +16121,11 @@
       </c>
       <c r="F72" s="59">
         <f t="shared" si="8"/>
-        <v>2820.4</v>
+        <v>2878.4</v>
       </c>
       <c r="G72" s="59">
         <f t="shared" si="9"/>
-        <v>2962.4</v>
+        <v>3074.4</v>
       </c>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
@@ -16152,11 +16149,11 @@
       </c>
       <c r="C73" s="60">
         <f t="shared" si="5"/>
-        <v>2476.3999999999996</v>
+        <v>2328.3999999999996</v>
       </c>
       <c r="D73" s="60">
         <f t="shared" si="6"/>
-        <v>2684.3999999999996</v>
+        <v>2612.3999999999996</v>
       </c>
       <c r="E73" s="60">
         <f t="shared" si="7"/>
@@ -16164,11 +16161,11 @@
       </c>
       <c r="F73" s="60">
         <f t="shared" si="8"/>
-        <v>3064.3999999999996</v>
+        <v>3132.3999999999996</v>
       </c>
       <c r="G73" s="60">
         <f t="shared" si="9"/>
-        <v>3236.3999999999996</v>
+        <v>3368.3999999999996</v>
       </c>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
@@ -16192,11 +16189,11 @@
       </c>
       <c r="C74" s="59">
         <f t="shared" si="5"/>
-        <v>2630.4</v>
+        <v>2462.4</v>
       </c>
       <c r="D74" s="59">
         <f t="shared" si="6"/>
-        <v>2868.4</v>
+        <v>2786.4</v>
       </c>
       <c r="E74" s="59">
         <f t="shared" si="7"/>
@@ -16204,11 +16201,11 @@
       </c>
       <c r="F74" s="59">
         <f t="shared" si="8"/>
-        <v>3308.4</v>
+        <v>3386.4</v>
       </c>
       <c r="G74" s="59">
         <f t="shared" si="9"/>
-        <v>3510.4</v>
+        <v>3662.4</v>
       </c>
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
@@ -16365,29 +16362,29 @@
       <c r="V80" s="4"/>
     </row>
     <row r="81" spans="2:22" ht="32" customHeight="1">
-      <c r="B81" s="92" t="s">
+      <c r="B81" s="91" t="s">
         <v>92</v>
       </c>
-      <c r="C81" s="92"/>
-      <c r="D81" s="92"/>
-      <c r="E81" s="92"/>
-      <c r="F81" s="92"/>
-      <c r="G81" s="92"/>
-      <c r="H81" s="92"/>
-      <c r="I81" s="92"/>
-      <c r="J81" s="92"/>
-      <c r="K81" s="92"/>
-      <c r="L81" s="92"/>
-      <c r="M81" s="92"/>
-      <c r="N81" s="92"/>
-      <c r="O81" s="92"/>
-      <c r="P81" s="92"/>
-      <c r="Q81" s="92"/>
-      <c r="R81" s="92"/>
-      <c r="S81" s="92"/>
-      <c r="T81" s="92"/>
-      <c r="U81" s="92"/>
-      <c r="V81" s="92"/>
+      <c r="C81" s="91"/>
+      <c r="D81" s="91"/>
+      <c r="E81" s="91"/>
+      <c r="F81" s="91"/>
+      <c r="G81" s="91"/>
+      <c r="H81" s="91"/>
+      <c r="I81" s="91"/>
+      <c r="J81" s="91"/>
+      <c r="K81" s="91"/>
+      <c r="L81" s="91"/>
+      <c r="M81" s="91"/>
+      <c r="N81" s="91"/>
+      <c r="O81" s="91"/>
+      <c r="P81" s="91"/>
+      <c r="Q81" s="91"/>
+      <c r="R81" s="91"/>
+      <c r="S81" s="91"/>
+      <c r="T81" s="91"/>
+      <c r="U81" s="91"/>
+      <c r="V81" s="91"/>
     </row>
     <row r="82" spans="2:22" ht="22" customHeight="1">
       <c r="B82" s="4"/>
@@ -16535,7 +16532,7 @@
       </c>
       <c r="J85" s="50">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R85)+(INDEX(Parameters!$J$13:$N$13,1,R85+1)-INDEX(Parameters!$J$13:$N$13,1,R85))*U85,INDEX(Parameters!$D$13:$H$13,1,R85)+(INDEX(Parameters!$D$13:$H$13,1,R85+1)-INDEX(Parameters!$D$13:$H$13,1,R85))*U85)</f>
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="K85" s="50">
         <f>IF('LSR Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R85)+(INDEX(Parameters!$D$14:$H$14,1,R85+1)-INDEX(Parameters!$D$14:$H$14,1,R85))*U85)</f>
@@ -16543,7 +16540,7 @@
       </c>
       <c r="L85" s="50">
         <f>I85+J85</f>
-        <v>2000</v>
+        <v>1600</v>
       </c>
       <c r="M85" s="50">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S85)+(INDEX(Parameters!$J$17:$N$17,1,S85+1)-INDEX(Parameters!$J$17:$N$17,1,S85))*V85,INDEX(Parameters!$D$17:$H$17,1,S85)+(INDEX(Parameters!$D$17:$H$17,1,S85+1)-INDEX(Parameters!$D$17:$H$17,1,S85))*V85)</f>
@@ -16621,7 +16618,7 @@
       </c>
       <c r="J86" s="52">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R86)+(INDEX(Parameters!$J$13:$N$13,1,R86+1)-INDEX(Parameters!$J$13:$N$13,1,R86))*U86,INDEX(Parameters!$D$13:$H$13,1,R86)+(INDEX(Parameters!$D$13:$H$13,1,R86+1)-INDEX(Parameters!$D$13:$H$13,1,R86))*U86)</f>
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="K86" s="52">
         <f>IF('LSR Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R86)+(INDEX(Parameters!$D$14:$H$14,1,R86+1)-INDEX(Parameters!$D$14:$H$14,1,R86))*U86)</f>
@@ -16629,7 +16626,7 @@
       </c>
       <c r="L86" s="52">
         <f>I86+J86</f>
-        <v>3155</v>
+        <v>2955</v>
       </c>
       <c r="M86" s="52">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S86)+(INDEX(Parameters!$J$17:$N$17,1,S86+1)-INDEX(Parameters!$J$17:$N$17,1,S86))*V86,INDEX(Parameters!$D$17:$H$17,1,S86)+(INDEX(Parameters!$D$17:$H$17,1,S86+1)-INDEX(Parameters!$D$17:$H$17,1,S86))*V86)</f>
@@ -16793,7 +16790,7 @@
       </c>
       <c r="J88" s="52">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R88)+(INDEX(Parameters!$J$13:$N$13,1,R88+1)-INDEX(Parameters!$J$13:$N$13,1,R88))*U88,INDEX(Parameters!$D$13:$H$13,1,R88)+(INDEX(Parameters!$D$13:$H$13,1,R88+1)-INDEX(Parameters!$D$13:$H$13,1,R88))*U88)</f>
-        <v>2600</v>
+        <v>2800</v>
       </c>
       <c r="K88" s="52">
         <f>IF('LSR Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R88)+(INDEX(Parameters!$D$14:$H$14,1,R88+1)-INDEX(Parameters!$D$14:$H$14,1,R88))*U88)</f>
@@ -16801,7 +16798,7 @@
       </c>
       <c r="L88" s="52">
         <f>I88+J88</f>
-        <v>5375</v>
+        <v>5575</v>
       </c>
       <c r="M88" s="52">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S88)+(INDEX(Parameters!$J$17:$N$17,1,S88+1)-INDEX(Parameters!$J$17:$N$17,1,S88))*V88,INDEX(Parameters!$D$17:$H$17,1,S88)+(INDEX(Parameters!$D$17:$H$17,1,S88+1)-INDEX(Parameters!$D$17:$H$17,1,S88))*V88)</f>
@@ -16879,7 +16876,7 @@
       </c>
       <c r="J89" s="50">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R89)+(INDEX(Parameters!$J$13:$N$13,1,R89+1)-INDEX(Parameters!$J$13:$N$13,1,R89))*U89,INDEX(Parameters!$D$13:$H$13,1,R89)+(INDEX(Parameters!$D$13:$H$13,1,R89+1)-INDEX(Parameters!$D$13:$H$13,1,R89))*U89)</f>
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="K89" s="50">
         <f>IF('LSR Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R89)+(INDEX(Parameters!$D$14:$H$14,1,R89+1)-INDEX(Parameters!$D$14:$H$14,1,R89))*U89)</f>
@@ -16887,7 +16884,7 @@
       </c>
       <c r="L89" s="50">
         <f>I89+J89</f>
-        <v>6440</v>
+        <v>6840</v>
       </c>
       <c r="M89" s="50">
         <f>IF('LSR Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S89)+(INDEX(Parameters!$J$17:$N$17,1,S89+1)-INDEX(Parameters!$J$17:$N$17,1,S89))*V89,INDEX(Parameters!$D$17:$H$17,1,S89)+(INDEX(Parameters!$D$17:$H$17,1,S89+1)-INDEX(Parameters!$D$17:$H$17,1,S89))*V89)</f>
@@ -18018,29 +18015,29 @@
       <c r="V120" s="4"/>
     </row>
     <row r="121" spans="2:22" ht="32" customHeight="1">
-      <c r="B121" s="92" t="s">
+      <c r="B121" s="91" t="s">
         <v>93</v>
       </c>
-      <c r="C121" s="92"/>
-      <c r="D121" s="92"/>
-      <c r="E121" s="92"/>
-      <c r="F121" s="92"/>
-      <c r="G121" s="92"/>
-      <c r="H121" s="92"/>
-      <c r="I121" s="92"/>
-      <c r="J121" s="92"/>
-      <c r="K121" s="92"/>
-      <c r="L121" s="92"/>
-      <c r="M121" s="92"/>
-      <c r="N121" s="92"/>
-      <c r="O121" s="92"/>
-      <c r="P121" s="92"/>
-      <c r="Q121" s="92"/>
-      <c r="R121" s="92"/>
-      <c r="S121" s="92"/>
-      <c r="T121" s="92"/>
-      <c r="U121" s="92"/>
-      <c r="V121" s="92"/>
+      <c r="C121" s="91"/>
+      <c r="D121" s="91"/>
+      <c r="E121" s="91"/>
+      <c r="F121" s="91"/>
+      <c r="G121" s="91"/>
+      <c r="H121" s="91"/>
+      <c r="I121" s="91"/>
+      <c r="J121" s="91"/>
+      <c r="K121" s="91"/>
+      <c r="L121" s="91"/>
+      <c r="M121" s="91"/>
+      <c r="N121" s="91"/>
+      <c r="O121" s="91"/>
+      <c r="P121" s="91"/>
+      <c r="Q121" s="91"/>
+      <c r="R121" s="91"/>
+      <c r="S121" s="91"/>
+      <c r="T121" s="91"/>
+      <c r="U121" s="91"/>
+      <c r="V121" s="91"/>
     </row>
     <row r="122" spans="2:22" ht="22" customHeight="1">
       <c r="B122" s="4"/>
@@ -18188,7 +18185,7 @@
       </c>
       <c r="J125" s="50">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R125)+(INDEX(Parameters!$J$13:$N$13,1,R125+1)-INDEX(Parameters!$J$13:$N$13,1,R125))*U125,INDEX(Parameters!$D$13:$H$13,1,R125)+(INDEX(Parameters!$D$13:$H$13,1,R125+1)-INDEX(Parameters!$D$13:$H$13,1,R125))*U125)</f>
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="K125" s="50">
         <f>IF('Full Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R125)+(INDEX(Parameters!$D$14:$H$14,1,R125+1)-INDEX(Parameters!$D$14:$H$14,1,R125))*U125)</f>
@@ -18196,7 +18193,7 @@
       </c>
       <c r="L125" s="50">
         <f>I125+J125</f>
-        <v>2000</v>
+        <v>1600</v>
       </c>
       <c r="M125" s="50">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S125)+(INDEX(Parameters!$J$17:$N$17,1,S125+1)-INDEX(Parameters!$J$17:$N$17,1,S125))*V125,INDEX(Parameters!$D$17:$H$17,1,S125)+(INDEX(Parameters!$D$17:$H$17,1,S125+1)-INDEX(Parameters!$D$17:$H$17,1,S125))*V125)</f>
@@ -18274,7 +18271,7 @@
       </c>
       <c r="J126" s="52">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R126)+(INDEX(Parameters!$J$13:$N$13,1,R126+1)-INDEX(Parameters!$J$13:$N$13,1,R126))*U126,INDEX(Parameters!$D$13:$H$13,1,R126)+(INDEX(Parameters!$D$13:$H$13,1,R126+1)-INDEX(Parameters!$D$13:$H$13,1,R126))*U126)</f>
-        <v>1400</v>
+        <v>1200</v>
       </c>
       <c r="K126" s="52">
         <f>IF('Full Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R126)+(INDEX(Parameters!$D$14:$H$14,1,R126+1)-INDEX(Parameters!$D$14:$H$14,1,R126))*U126)</f>
@@ -18282,7 +18279,7 @@
       </c>
       <c r="L126" s="52">
         <f>I126+J126</f>
-        <v>3155</v>
+        <v>2955</v>
       </c>
       <c r="M126" s="52">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S126)+(INDEX(Parameters!$J$17:$N$17,1,S126+1)-INDEX(Parameters!$J$17:$N$17,1,S126))*V126,INDEX(Parameters!$D$17:$H$17,1,S126)+(INDEX(Parameters!$D$17:$H$17,1,S126+1)-INDEX(Parameters!$D$17:$H$17,1,S126))*V126)</f>
@@ -18446,7 +18443,7 @@
       </c>
       <c r="J128" s="52">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R128)+(INDEX(Parameters!$J$13:$N$13,1,R128+1)-INDEX(Parameters!$J$13:$N$13,1,R128))*U128,INDEX(Parameters!$D$13:$H$13,1,R128)+(INDEX(Parameters!$D$13:$H$13,1,R128+1)-INDEX(Parameters!$D$13:$H$13,1,R128))*U128)</f>
-        <v>2600</v>
+        <v>2800</v>
       </c>
       <c r="K128" s="52">
         <f>IF('Full Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R128)+(INDEX(Parameters!$D$14:$H$14,1,R128+1)-INDEX(Parameters!$D$14:$H$14,1,R128))*U128)</f>
@@ -18454,7 +18451,7 @@
       </c>
       <c r="L128" s="52">
         <f>I128+J128</f>
-        <v>5375</v>
+        <v>5575</v>
       </c>
       <c r="M128" s="52">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S128)+(INDEX(Parameters!$J$17:$N$17,1,S128+1)-INDEX(Parameters!$J$17:$N$17,1,S128))*V128,INDEX(Parameters!$D$17:$H$17,1,S128)+(INDEX(Parameters!$D$17:$H$17,1,S128+1)-INDEX(Parameters!$D$17:$H$17,1,S128))*V128)</f>
@@ -18532,7 +18529,7 @@
       </c>
       <c r="J129" s="50">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R129)+(INDEX(Parameters!$J$13:$N$13,1,R129+1)-INDEX(Parameters!$J$13:$N$13,1,R129))*U129,INDEX(Parameters!$D$13:$H$13,1,R129)+(INDEX(Parameters!$D$13:$H$13,1,R129+1)-INDEX(Parameters!$D$13:$H$13,1,R129))*U129)</f>
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="K129" s="50">
         <f>IF('Full Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R129)+(INDEX(Parameters!$D$14:$H$14,1,R129+1)-INDEX(Parameters!$D$14:$H$14,1,R129))*U129)</f>
@@ -18540,7 +18537,7 @@
       </c>
       <c r="L129" s="50">
         <f>I129+J129</f>
-        <v>6440</v>
+        <v>6840</v>
       </c>
       <c r="M129" s="50">
         <f>IF('Full Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S129)+(INDEX(Parameters!$J$17:$N$17,1,S129+1)-INDEX(Parameters!$J$17:$N$17,1,S129))*V129,INDEX(Parameters!$D$17:$H$17,1,S129)+(INDEX(Parameters!$D$17:$H$17,1,S129+1)-INDEX(Parameters!$D$17:$H$17,1,S129))*V129)</f>
@@ -19373,11 +19370,11 @@
       </c>
       <c r="C146" s="59">
         <f t="shared" si="15"/>
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="D146" s="59">
         <f t="shared" si="16"/>
-        <v>1072.4000000000001</v>
+        <v>1070.4000000000001</v>
       </c>
       <c r="E146" s="59">
         <f t="shared" si="17"/>
@@ -19428,11 +19425,11 @@
       </c>
       <c r="C147" s="60">
         <f t="shared" si="15"/>
-        <v>836</v>
+        <v>808</v>
       </c>
       <c r="D147" s="60">
         <f t="shared" si="16"/>
-        <v>1230.1500000000001</v>
+        <v>1218.1500000000001</v>
       </c>
       <c r="E147" s="60">
         <f t="shared" si="17"/>
@@ -19440,11 +19437,11 @@
       </c>
       <c r="F147" s="60">
         <f t="shared" si="18"/>
-        <v>1934.75</v>
+        <v>1942.75</v>
       </c>
       <c r="G147" s="60">
         <f t="shared" si="19"/>
-        <v>2245.1999999999998</v>
+        <v>2257.1999999999998</v>
       </c>
       <c r="H147" s="60">
         <f t="shared" si="20"/>
@@ -19483,11 +19480,11 @@
       </c>
       <c r="C148" s="59">
         <f t="shared" si="15"/>
-        <v>936</v>
+        <v>888</v>
       </c>
       <c r="D148" s="59">
         <f t="shared" si="16"/>
-        <v>1387.9</v>
+        <v>1365.9</v>
       </c>
       <c r="E148" s="59">
         <f t="shared" si="17"/>
@@ -19495,11 +19492,11 @@
       </c>
       <c r="F148" s="59">
         <f t="shared" si="18"/>
-        <v>2203.5</v>
+        <v>2221.5</v>
       </c>
       <c r="G148" s="59">
         <f t="shared" si="19"/>
-        <v>2567.1999999999998</v>
+        <v>2599.1999999999998</v>
       </c>
       <c r="H148" s="59">
         <f t="shared" si="20"/>
@@ -19538,11 +19535,11 @@
       </c>
       <c r="C149" s="60">
         <f t="shared" si="15"/>
-        <v>1036</v>
+        <v>968</v>
       </c>
       <c r="D149" s="60">
         <f t="shared" si="16"/>
-        <v>1545.65</v>
+        <v>1513.65</v>
       </c>
       <c r="E149" s="60">
         <f t="shared" si="17"/>
@@ -19550,11 +19547,11 @@
       </c>
       <c r="F149" s="60">
         <f t="shared" si="18"/>
-        <v>2472.25</v>
+        <v>2500.25</v>
       </c>
       <c r="G149" s="60">
         <f t="shared" si="19"/>
-        <v>2889.2</v>
+        <v>2941.2</v>
       </c>
       <c r="H149" s="60">
         <f t="shared" si="20"/>
@@ -19593,11 +19590,11 @@
       </c>
       <c r="C150" s="59">
         <f t="shared" si="15"/>
-        <v>1136.0000000000002</v>
+        <v>1048.0000000000002</v>
       </c>
       <c r="D150" s="59">
         <f t="shared" si="16"/>
-        <v>1703.4</v>
+        <v>1661.4</v>
       </c>
       <c r="E150" s="59">
         <f t="shared" si="17"/>
@@ -19605,11 +19602,11 @@
       </c>
       <c r="F150" s="59">
         <f t="shared" si="18"/>
-        <v>2741</v>
+        <v>2779</v>
       </c>
       <c r="G150" s="59">
         <f t="shared" si="19"/>
-        <v>3211.2000000000003</v>
+        <v>3283.2000000000007</v>
       </c>
       <c r="H150" s="59">
         <f t="shared" si="20"/>
@@ -19648,11 +19645,11 @@
       </c>
       <c r="C151" s="60">
         <f t="shared" si="15"/>
-        <v>1236</v>
+        <v>1128</v>
       </c>
       <c r="D151" s="60">
         <f t="shared" si="16"/>
-        <v>1861.1499999999999</v>
+        <v>1809.1499999999999</v>
       </c>
       <c r="E151" s="60">
         <f t="shared" si="17"/>
@@ -19660,11 +19657,11 @@
       </c>
       <c r="F151" s="60">
         <f t="shared" si="18"/>
-        <v>3009.75</v>
+        <v>3057.75</v>
       </c>
       <c r="G151" s="60">
         <f t="shared" si="19"/>
-        <v>3533.2</v>
+        <v>3625.2</v>
       </c>
       <c r="H151" s="60">
         <f t="shared" si="20"/>
@@ -19703,11 +19700,11 @@
       </c>
       <c r="C152" s="59">
         <f t="shared" si="15"/>
-        <v>1336</v>
+        <v>1208</v>
       </c>
       <c r="D152" s="59">
         <f t="shared" si="16"/>
-        <v>2018.9</v>
+        <v>1956.9</v>
       </c>
       <c r="E152" s="59">
         <f t="shared" si="17"/>
@@ -19715,11 +19712,11 @@
       </c>
       <c r="F152" s="59">
         <f t="shared" si="18"/>
-        <v>3278.5</v>
+        <v>3336.5</v>
       </c>
       <c r="G152" s="59">
         <f t="shared" si="19"/>
-        <v>3855.2000000000003</v>
+        <v>3967.2000000000003</v>
       </c>
       <c r="H152" s="59">
         <f t="shared" si="20"/>
@@ -19758,11 +19755,11 @@
       </c>
       <c r="C153" s="60">
         <f t="shared" si="15"/>
-        <v>1436</v>
+        <v>1288</v>
       </c>
       <c r="D153" s="60">
         <f t="shared" si="16"/>
-        <v>2176.6499999999996</v>
+        <v>2104.6499999999996</v>
       </c>
       <c r="E153" s="60">
         <f t="shared" si="17"/>
@@ -19770,11 +19767,11 @@
       </c>
       <c r="F153" s="60">
         <f t="shared" si="18"/>
-        <v>3547.25</v>
+        <v>3615.25</v>
       </c>
       <c r="G153" s="60">
         <f t="shared" si="19"/>
-        <v>4177.2</v>
+        <v>4309.2</v>
       </c>
       <c r="H153" s="60">
         <f t="shared" si="20"/>
@@ -19813,11 +19810,11 @@
       </c>
       <c r="C154" s="59">
         <f t="shared" si="15"/>
-        <v>1536</v>
+        <v>1368</v>
       </c>
       <c r="D154" s="59">
         <f t="shared" si="16"/>
-        <v>2334.4</v>
+        <v>2252.4</v>
       </c>
       <c r="E154" s="59">
         <f t="shared" si="17"/>
@@ -19825,11 +19822,11 @@
       </c>
       <c r="F154" s="59">
         <f t="shared" si="18"/>
-        <v>3816</v>
+        <v>3894</v>
       </c>
       <c r="G154" s="59">
         <f t="shared" si="19"/>
-        <v>4499.2</v>
+        <v>4651.2</v>
       </c>
       <c r="H154" s="59">
         <f t="shared" si="20"/>
@@ -19932,29 +19929,29 @@
       <c r="V157" s="4"/>
     </row>
     <row r="161" spans="2:22" ht="32" customHeight="1">
-      <c r="B161" s="93" t="s">
+      <c r="B161" s="92" t="s">
         <v>94</v>
       </c>
-      <c r="C161" s="93"/>
-      <c r="D161" s="93"/>
-      <c r="E161" s="93"/>
-      <c r="F161" s="93"/>
-      <c r="G161" s="93"/>
-      <c r="H161" s="93"/>
-      <c r="I161" s="93"/>
-      <c r="J161" s="93"/>
-      <c r="K161" s="93"/>
-      <c r="L161" s="93"/>
-      <c r="M161" s="93"/>
-      <c r="N161" s="93"/>
-      <c r="O161" s="93"/>
-      <c r="P161" s="93"/>
-      <c r="Q161" s="93"/>
-      <c r="R161" s="93"/>
-      <c r="S161" s="93"/>
-      <c r="T161" s="93"/>
-      <c r="U161" s="93"/>
-      <c r="V161" s="93"/>
+      <c r="C161" s="92"/>
+      <c r="D161" s="92"/>
+      <c r="E161" s="92"/>
+      <c r="F161" s="92"/>
+      <c r="G161" s="92"/>
+      <c r="H161" s="92"/>
+      <c r="I161" s="92"/>
+      <c r="J161" s="92"/>
+      <c r="K161" s="92"/>
+      <c r="L161" s="92"/>
+      <c r="M161" s="92"/>
+      <c r="N161" s="92"/>
+      <c r="O161" s="92"/>
+      <c r="P161" s="92"/>
+      <c r="Q161" s="92"/>
+      <c r="R161" s="92"/>
+      <c r="S161" s="92"/>
+      <c r="T161" s="92"/>
+      <c r="U161" s="92"/>
+      <c r="V161" s="92"/>
     </row>
     <row r="164" spans="2:22" ht="44" customHeight="1">
       <c r="B164" s="61" t="s">
@@ -20053,7 +20050,7 @@
       </c>
       <c r="J165" s="63">
         <f>IF(Calculator!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R165)+(INDEX(Parameters!$J$13:$N$13,1,R165+1)-INDEX(Parameters!$J$13:$N$13,1,R165))*U165,INDEX(Parameters!$D$13:$H$13,1,R165)+(INDEX(Parameters!$D$13:$H$13,1,R165+1)-INDEX(Parameters!$D$13:$H$13,1,R165))*U165)</f>
-        <v>2240</v>
+        <v>2320</v>
       </c>
       <c r="K165" s="63">
         <f>IF(Calculator!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R165)+(INDEX(Parameters!$D$14:$H$14,1,R165+1)-INDEX(Parameters!$D$14:$H$14,1,R165))*U165)</f>
@@ -20061,7 +20058,7 @@
       </c>
       <c r="L165" s="63">
         <f>I165+J165</f>
-        <v>4520</v>
+        <v>4600</v>
       </c>
       <c r="M165" s="63">
         <f>IF(Calculator!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S165)+(INDEX(Parameters!$J$17:$N$17,1,S165+1)-INDEX(Parameters!$J$17:$N$17,1,S165))*V165,INDEX(Parameters!$D$17:$H$17,1,S165)+(INDEX(Parameters!$D$17:$H$17,1,S165+1)-INDEX(Parameters!$D$17:$H$17,1,S165))*V165)</f>

</xml_diff>